<commit_message>
fix(admin): header-only sample sheet and correct quarter format hint
Remove the illustrative sample row from the downloadable template so it
contains only the column headers. Fix the Quarter field hint to suggest
the correct space-separated format (Q1 FY27) instead of the hyphenated
Q1-FY27, matching the input placeholder.
</commit_message>
<xml_diff>
--- a/public/research-sheet-template.xlsx
+++ b/public/research-sheet-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,32 +422,9 @@
         <v>Note</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Example Industries Ltd</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Capital Goods</v>
-      </c>
-      <c r="C2">
-        <v>12345.67</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Tier 1</v>
-      </c>
-      <c r="E2" t="str">
-        <v>EXAMPLE</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Positive</v>
-      </c>
-      <c r="G2" t="str">
-        <v>One-line, plain-English view for this quarter.</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>